<commit_message>
fix: harden position reconciliation persistence
</commit_message>
<xml_diff>
--- a/assets/中台网关原始入账订单.xlsx
+++ b/assets/中台网关原始入账订单.xlsx
@@ -563,8 +563,7 @@
     <col min="15" max="15" width="28" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="20" style="1" customWidth="1"/>
-    <col min="18" max="18" width="14" style="1" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="18" max="19" width="14" style="1" customWidth="1"/>
     <col min="20" max="20" width="18" style="1" customWidth="1"/>
     <col min="21" max="21" width="14" customWidth="1"/>
     <col min="22" max="22" width="16" style="1" customWidth="1"/>
@@ -640,7 +639,7 @@
       <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="2" t="s">

</xml_diff>